<commit_message>
Add clickable profile links to the Chart tab
Appends a compact Name/Niche/Profile-Link table to the bottom of the
Chart tab so the graph view is self-contained with direct click-through
links, alongside the existing niche and follower-count bars.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KMn3Gx6a7DZRK9hu7NkZ3P
</commit_message>
<xml_diff>
--- a/nh_creator_scout/NH_TikTok_EcommerceTrading_New25.xlsx
+++ b/nh_creator_scout/NH_TikTok_EcommerceTrading_New25.xlsx
@@ -106,7 +106,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -133,6 +133,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1982,7 +1986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2215,7 +2219,571 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>All 25 Profiles</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Niche</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Profile Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>سهل مهدي / Sahel Mahdi</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@sahelmahdi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>د. عبدالكريم عنف / Dr. Abdulkarim Anaf</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@anafabdulkareem</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>LLC4ARAB</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@llc4arab</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>ابراهيم البحراوي / Ibrahim Al-Bahrawy</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>https://bhrawy.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>علاء الحسن / Alaa Al-Hassan</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>https://alaaalhasan.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>أحمد مطر / Ahmed Matar</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>https://ahmedmtr.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>@ifast.sa</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@ifast.sa</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>فهيد الفهيد / Fahad Al-Fahad</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@fh_afiliate0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>بيان لنجكاوي / Bayan Lanjakawi</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>No confirmed handle — see Creators tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>بزنس فاطمة / Fatemah Business</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@fatemahbusiness</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>عالية العالي / Aliya Al-Ali (No Added Sugar)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>E-commerce</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/noaddedsugar.me/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>أبو ريان / Abu Rayan</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.snapchat.com/@aaboryan</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>أبو إبراهيم / Abu Ibrahim ("Wolfe Wave")</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@wolfe_wave</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>مكهرب الأسهم ("أبو عبدالله") / Mkahrib Al-Ashom</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/mokhrepashom</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>خبير أسهم / Khabeer Ashom ("Stock Expert")</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/khabeer999</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>قناة تاسي / TASI_y</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@tasi_y</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>أبو نوره / KsaTrader (Abu Nourah)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/KsaTrader</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>محمد الميموني / Mohammad Al-Maimoni</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/mohammad_fx</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>شؤون الأسهم / Stock Affairs</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/Stock_Affairs</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>د. عبدالله المزراقي / Dr. Abdullah Al-Mezraqi</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@dr.mezraqi</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>USA Stock Hunter (صائد الأسهم الأمريكية)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@usastockhunter</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>أكاديمية بندر المحسن المالية / Bandar Al-Mohsin Financial Academy</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>https://x.com/BAlmohsin1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Atradez ("Ahmed")</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@atradez</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>صالح القحطاني / Saleh Al-Qahtani</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.snapchat.com/@s-qht11</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>محمد الحديثي / Mohammed Al-Hudaithi</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@mhmh1199</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId24"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>